<commit_message>
Sync ISM2411 DataCamp assignment list with actual course/due-date data
Update the front page, syllabus, README, and Canvas cartridge manifest to
the real 5 required + 2 extra-credit courses, matching what's actually
assigned in DataCamp for Classrooms. Fix the due-dates spreadsheet to
match: drop the 3 courses that were never actually required, and move
the 2 extra-credit courses to their real Nov 29 due date.

Bumps the ism2411 submodule pointer for the matching website changes.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WFo17bHe1nRycYkg8Zak3c
</commit_message>
<xml_diff>
--- a/schedules/ism2411_due_dates.xlsx
+++ b/schedules/ism2411_due_dates.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="15120" windowHeight="18980" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ISM2411 Due Dates" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,15 +12,14 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ISM2411 Due Dates'!$A$1:$G$18</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -33,12 +31,16 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="6">
@@ -50,26 +52,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3A5F"/>
-        <bgColor rgb="001F3A5F"/>
+        <fgColor rgb="FF1F3A5F"/>
+        <bgColor rgb="FF1F3A5F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FBF8ED"/>
-        <bgColor rgb="00FBF8ED"/>
+        <fgColor rgb="FFFBF8ED"/>
+        <bgColor rgb="FFFBF8ED"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F7E4DF"/>
-        <bgColor rgb="00F7E4DF"/>
+        <fgColor rgb="FFF7E4DF"/>
+        <bgColor rgb="FFF7E4DF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E9F1EC"/>
-        <bgColor rgb="00E9F1EC"/>
+        <fgColor rgb="FFE9F1EC"/>
+        <bgColor rgb="FFE9F1EC"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,23 +85,24 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00C7D2DC"/>
+        <color rgb="FFC7D2DC"/>
       </left>
       <right style="thin">
-        <color rgb="00C7D2DC"/>
+        <color rgb="FFC7D2DC"/>
       </right>
       <top style="thin">
-        <color rgb="00C7D2DC"/>
+        <color rgb="FFC7D2DC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00C7D2DC"/>
+        <color rgb="FFC7D2DC"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -107,7 +110,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -119,7 +122,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -131,7 +134,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -143,7 +146,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -159,9 +162,21 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -525,13 +540,12 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="4" max="5"/>
     <col width="42" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
@@ -574,7 +588,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" s="23" t="n">
         <v>46264</v>
       </c>
       <c r="B2" s="4" t="n">
@@ -590,12 +604,12 @@
           <t>Quiz 1</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr"/>
-      <c r="F2" s="5" t="inlineStr"/>
-      <c r="G2" s="6" t="inlineStr"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="5" t="n"/>
+      <c r="G2" s="6" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="n">
+      <c r="A3" s="24" t="n">
         <v>46271</v>
       </c>
       <c r="B3" s="8" t="n">
@@ -621,10 +635,10 @@
           <t>DataCamp: Introduction to Python (Required)</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr"/>
+      <c r="G3" s="10" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="23" t="n">
         <v>46278</v>
       </c>
       <c r="B4" s="4" t="n">
@@ -645,11 +659,11 @@
           <t>Lab 3</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="6" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="24" t="n">
         <v>46285</v>
       </c>
       <c r="B5" s="8" t="n">
@@ -675,10 +689,10 @@
           <t>DataCamp: Intermediate Python (Required)</t>
         </is>
       </c>
-      <c r="G5" s="10" t="inlineStr"/>
+      <c r="G5" s="10" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="23" t="n">
         <v>46292</v>
       </c>
       <c r="B6" s="4" t="n">
@@ -699,11 +713,11 @@
           <t>Lab 5</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="24" t="n">
         <v>46299</v>
       </c>
       <c r="B7" s="8" t="n">
@@ -729,10 +743,10 @@
           <t>DataCamp: Python Toolbox (Required)</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr"/>
+      <c r="G7" s="10" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="24" t="n">
         <v>46306</v>
       </c>
       <c r="B8" s="8" t="n">
@@ -758,10 +772,10 @@
           <t>DataCamp: Writing Functions in Python (Required)</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr"/>
+      <c r="G8" s="10" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="23" t="n">
         <v>46313</v>
       </c>
       <c r="B9" s="4" t="n">
@@ -782,11 +796,11 @@
           <t>Lab 8</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr"/>
-      <c r="G9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="11" t="n">
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="25" t="n">
         <v>46320</v>
       </c>
       <c r="B10" s="12" t="n">
@@ -797,9 +811,9 @@
           <t>Midterm Exam</t>
         </is>
       </c>
-      <c r="D10" s="12" t="inlineStr"/>
-      <c r="E10" s="12" t="inlineStr"/>
-      <c r="F10" s="13" t="inlineStr"/>
+      <c r="D10" s="12" t="n"/>
+      <c r="E10" s="12" t="n"/>
+      <c r="F10" s="13" t="n"/>
       <c r="G10" s="14" t="inlineStr">
         <is>
           <t>Midterm Exam (in-class, 75 min)</t>
@@ -807,7 +821,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="24" t="n">
         <v>46327</v>
       </c>
       <c r="B11" s="8" t="n">
@@ -830,42 +844,38 @@
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>DataCamp: Data Types for Data Science (Required)</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="inlineStr"/>
+          <t>DataCamp: Data Types in Python (Required)</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="n">
+      <c r="A12" s="23" t="n">
         <v>46334</v>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Dictionaries</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Quiz 11</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Lab 11</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>DataCamp: Working with Dictionaries (Required)</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="inlineStr"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="6" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="23" t="n">
         <v>46341</v>
       </c>
       <c r="B13" s="4" t="n">
@@ -886,40 +896,36 @@
           <t>Lab 12</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr"/>
-      <c r="G13" s="6" t="inlineStr"/>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n">
+      <c r="A14" s="23" t="n">
         <v>46348</v>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Intro to pandas</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Quiz 13</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Lab 13</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
-        <is>
-          <t>DataCamp: Introduction to pandas (Required)</t>
-        </is>
-      </c>
-      <c r="G14" s="10" t="inlineStr"/>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="6" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n">
+      <c r="A15" s="24" t="n">
         <v>46355</v>
       </c>
       <c r="B15" s="8" t="n">
@@ -942,63 +948,59 @@
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>DataCamp: Data Manipulation with pandas (Required)</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="inlineStr"/>
+          <t>DataCamp: Joining Data with pandas (Bonus)</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="n">
+      <c r="A16" s="24" t="n">
+        <v>46355</v>
+      </c>
+      <c r="B16" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Data Cleaning &amp; Descriptive Stats</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>DataCamp: Introduction to Data Visualization with Matplotlib (Bonus)</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="n">
         <v>46362</v>
       </c>
-      <c r="B16" s="8" t="n">
+      <c r="B17" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Grouping &amp; Visualization</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Quiz 15</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Lab 15</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>DataCamp: Joining Data with pandas (Bonus)</t>
-        </is>
-      </c>
-      <c r="G16" s="10" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="n">
-        <v>46362</v>
-      </c>
-      <c r="B17" s="8" t="n">
-        <v>15</v>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>Grouping &amp; Visualization</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr"/>
-      <c r="E17" s="8" t="inlineStr"/>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>DataCamp: Introduction to Data Visualization with Matplotlib (Bonus)</t>
-        </is>
-      </c>
-      <c r="G17" s="10" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="15" t="n">
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="6" t="n"/>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="26" t="n">
         <v>46369</v>
       </c>
       <c r="B18" s="16" t="n">
@@ -1009,9 +1011,9 @@
           <t>Capstone Project</t>
         </is>
       </c>
-      <c r="D18" s="16" t="inlineStr"/>
-      <c r="E18" s="16" t="inlineStr"/>
-      <c r="F18" s="17" t="inlineStr"/>
+      <c r="D18" s="16" t="n"/>
+      <c r="E18" s="16" t="n"/>
+      <c r="F18" s="17" t="n"/>
       <c r="G18" s="18" t="inlineStr">
         <is>
           <t>Capstone Project due + live presentation</t>
@@ -1031,7 +1033,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>

</xml_diff>